<commit_message>
Adventure: split sidebar variant and single-slide slider spacing, as on wknd.site
Three adventure pages (yosemite, tahoe, west coast cycling) author their
sidebar as grid columns on the source, which lays out differently:
- importer: wknd-adventure marks such sidebars, and wknd-sections now
  accepts a page-specific extra section style from a template
  transformer (data-section-style), giving "sidebar, split"
- styles.css: split sidebar shows the facts and "Share this Adventure"
  side by side below 1025px (7 / 5 columns on phones, 9 / 3 from 768px);
  those pages set the title and tabs 14px from the edge and inset the
  desktop breadcrumb and sidebar by 14px
- carousel-hero (mini): one slide keeps the 26px dot row WKND shows

Home, magazine and all articles re-import byte-identical.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure.report.xlsx
+++ b/tools/importer/reports/import-adventure.report.xlsx
@@ -58,7 +58,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-27T17:14:23.734Z</t>
+    <t>2026-09-28T05:59:23.894Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -82,7 +82,7 @@
     <t>magazine</t>
   </si>
   <si>
-    <t>2026-09-27T17:14:29.373Z</t>
+    <t>2026-09-28T05:59:30.781Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -106,7 +106,7 @@
     <t>adventure</t>
   </si>
   <si>
-    <t>2026-09-28T05:39:03.274Z</t>
+    <t>2026-09-28T06:00:03.835Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -121,7 +121,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-28T05:39:09.259Z</t>
+    <t>2026-09-28T06:00:09.686Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -136,7 +136,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-28T05:39:15.191Z</t>
+    <t>2026-09-28T06:00:13.943Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -151,7 +151,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-28T05:39:22.338Z</t>
+    <t>2026-09-28T06:00:20.503Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -169,7 +169,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-28T05:39:28.287Z</t>
+    <t>2026-09-28T06:00:25.718Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -184,7 +184,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-28T05:39:33.017Z</t>
+    <t>2026-09-28T06:00:31.902Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -208,7 +208,7 @@
     <t>article</t>
   </si>
   <si>
-    <t>2026-09-27T17:57:34.382Z</t>
+    <t>2026-09-28T05:59:42.238Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -226,7 +226,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-27T17:57:42.113Z</t>
+    <t>2026-09-28T05:59:48.423Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -241,7 +241,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-27T17:57:47.754Z</t>
+    <t>2026-09-28T05:59:52.683Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -259,7 +259,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-27T17:57:53.581Z</t>
+    <t>2026-09-28T05:59:56.697Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -277,7 +277,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-27T17:57:29.061Z</t>
+    <t>2026-09-28T05:59:37.701Z</t>
   </si>
   <si>
     <t>Western Australia</t>

</xml_diff>

<commit_message>
Adventure: keep image captions in tabs, 48px before the footer
- tabs parser: an image's caption (WKND image title, shown under the
  image on yosemite and tahoe) was dropped; it now becomes an italic
  paragraph after the image, styled as the WKND caption in tabs.css
  (replaces the opening-image spacing rule, which was the caption's space)
- adventure pages: 48px between the tabs and the footer, as on the source

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure.report.xlsx
+++ b/tools/importer/reports/import-adventure.report.xlsx
@@ -106,7 +106,7 @@
     <t>adventure</t>
   </si>
   <si>
-    <t>2026-09-28T06:00:03.835Z</t>
+    <t>2026-09-28T06:11:14.621Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -121,7 +121,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-28T06:00:09.686Z</t>
+    <t>2026-09-28T06:11:19.916Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -136,7 +136,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-28T06:00:13.943Z</t>
+    <t>2026-09-28T06:11:26.660Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -151,7 +151,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-28T06:00:20.503Z</t>
+    <t>2026-09-28T06:11:32.880Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -169,7 +169,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-28T06:00:25.718Z</t>
+    <t>2026-09-28T06:11:37.918Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -184,7 +184,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-28T06:00:31.902Z</t>
+    <t>2026-09-28T06:11:42.534Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>

</xml_diff>

<commit_message>
Bulk import: cycling-southern-utah and bali-surf-camp on the adventure template
Both match the approved adventure template (image slider, facts, three
tabs; grid-column sidebar -> "sidebar, split"). The six existing
adventure pages re-import byte-identical.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure.report.xlsx
+++ b/tools/importer/reports/import-adventure.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="122">
   <si>
     <t>_reportFile</t>
   </si>
@@ -67,12 +67,75 @@
     <t>https://wknd.site/us/en.html</t>
   </si>
   <si>
+    <t>us/en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>["cards","cards","cards","cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us/en/about-us</t>
+  </si>
+  <si>
+    <t>about</t>
+  </si>
+  <si>
+    <t>2026-09-28T06:49:29.123Z</t>
+  </si>
+  <si>
+    <t>About Us</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/about-us.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures.report.json</t>
+  </si>
+  <si>
+    <t>["hero-teaser","cards-article"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures</t>
+  </si>
+  <si>
+    <t>adventure-listing</t>
+  </si>
+  <si>
+    <t>2026-09-28T06:21:34.372Z</t>
+  </si>
+  <si>
+    <t>Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures.html</t>
+  </si>
+  <si>
+    <t>us/en/faqs.report.json</t>
+  </si>
+  <si>
+    <t>["accordion"]</t>
+  </si>
+  <si>
+    <t>us/en/faqs</t>
+  </si>
+  <si>
+    <t>faq</t>
+  </si>
+  <si>
+    <t>2026-09-28T06:37:54.159Z</t>
+  </si>
+  <si>
+    <t>FAQs</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
     <t>us/en/magazine.report.json</t>
   </si>
   <si>
-    <t>[]</t>
-  </si>
-  <si>
     <t>["columns-featured","cards-article","cards-article","cards-article"]</t>
   </si>
   <si>
@@ -91,22 +154,37 @@
     <t>https://wknd.site/us/en/magazine.html</t>
   </si>
   <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["carousel-hero","cards-related","tabs"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventure</t>
+  </si>
+  <si>
+    <t>2026-09-28T07:04:26.853Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
     <t>us/en/adventures/climbing-new-zealand.report.json</t>
   </si>
   <si>
     <t>["What to Bring — empty alt, used tab label"]</t>
   </si>
   <si>
-    <t>["carousel-hero","cards-related","tabs"]</t>
-  </si>
-  <si>
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>adventure</t>
-  </si>
-  <si>
-    <t>2026-09-28T06:11:14.621Z</t>
+    <t>2026-09-28T07:03:49.543Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -115,13 +193,28 @@
     <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
   </si>
   <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-28T07:04:21.005Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
     <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
   </si>
   <si>
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-28T06:11:19.916Z</t>
+    <t>2026-09-28T07:03:54.583Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -136,7 +229,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-28T06:11:26.660Z</t>
+    <t>2026-09-28T07:03:59.517Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -151,7 +244,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-28T06:11:32.880Z</t>
+    <t>2026-09-28T07:04:05.046Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -169,7 +262,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-28T06:11:37.918Z</t>
+    <t>2026-09-28T07:04:10.327Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -184,7 +277,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-28T06:11:42.534Z</t>
+    <t>2026-09-28T07:04:15.716Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -672,12 +765,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
     <col min="4" max="4" width="43" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="8" width="33" customWidth="1"/>
     <col min="9" max="9" width="50" customWidth="1"/>
@@ -775,39 +868,39 @@
         <v>26</v>
       </c>
       <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
         <v>27</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>28</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
         <v>29</v>
       </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>30</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>31</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>32</v>
-      </c>
-      <c r="I4" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
         <v>35</v>
@@ -816,259 +909,259 @@
         <v>13</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6" t="s">
         <v>13</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H6" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="I6" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
         <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
         <v>13</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="G7" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="H7" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="I7" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
         <v>50</v>
       </c>
-      <c r="C8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" t="s">
-        <v>51</v>
-      </c>
-      <c r="E8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" t="s">
-        <v>30</v>
-      </c>
       <c r="G8" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="H8" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="I8" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
         <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E9" t="s">
         <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="G9" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="H9" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="I9" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E10" t="s">
         <v>13</v>
       </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" t="s">
         <v>13</v>
       </c>
       <c r="F11" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
         <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="D12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E12" t="s">
         <v>13</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="D13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E13" t="s">
         <v>13</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>86</v>
+        <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="D14" t="s">
         <v>87</v>
@@ -1077,7 +1170,7 @@
         <v>13</v>
       </c>
       <c r="F14" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G14" t="s">
         <v>88</v>
@@ -1087,6 +1180,151 @@
       </c>
       <c r="I14" t="s">
         <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>95</v>
+      </c>
+      <c r="G15" t="s">
+        <v>96</v>
+      </c>
+      <c r="H15" t="s">
+        <v>97</v>
+      </c>
+      <c r="I15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" t="s">
+        <v>101</v>
+      </c>
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G16" t="s">
+        <v>102</v>
+      </c>
+      <c r="H16" t="s">
+        <v>103</v>
+      </c>
+      <c r="I16" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>105</v>
+      </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" t="s">
+        <v>106</v>
+      </c>
+      <c r="E17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" t="s">
+        <v>107</v>
+      </c>
+      <c r="H17" t="s">
+        <v>108</v>
+      </c>
+      <c r="I17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B18" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" t="s">
+        <v>93</v>
+      </c>
+      <c r="D18" t="s">
+        <v>112</v>
+      </c>
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H18" t="s">
+        <v>114</v>
+      </c>
+      <c r="I18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" t="s">
+        <v>117</v>
+      </c>
+      <c r="C19" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" t="s">
+        <v>118</v>
+      </c>
+      <c r="E19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" t="s">
+        <v>95</v>
+      </c>
+      <c r="G19" t="s">
+        <v>119</v>
+      </c>
+      <c r="H19" t="s">
+        <v>120</v>
+      </c>
+      <c r="I19" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>